<commit_message>
Fix Mama Busi and Jewellery stock sheets
Mama Busi: ironing board covers, peg bags, peg cabin hooks (15 products)
- Removed mats (wrong category) and fashion items
- Removed mats_stock.csv

Jewellery: 98 products with selling prices from WC
- Notes column prompts to fill in cost prices

https://claude.ai/code/session_012ekkvYAvXX5Y4AhF5m3cWa
</commit_message>
<xml_diff>
--- a/woocommerce/suppliers/mama_busi/stock_sheet.xlsx
+++ b/woocommerce/suppliers/mama_busi/stock_sheet.xlsx
@@ -110,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -127,7 +127,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -136,13 +136,10 @@
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -151,10 +148,7 @@
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -531,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S74"/>
+  <dimension ref="A1:S67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -558,7 +552,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Mama Busi (Mats &amp; Rugs) — Stock Sheet   (updated: 2026-03-12)</t>
+          <t>Mama Busi — Stock Sheet   (updated: 2026-03-12)</t>
         </is>
       </c>
     </row>
@@ -661,24 +655,34 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr"/>
-      <c r="B3" s="4" t="inlineStr"/>
-      <c r="C3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>9902056295991</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>10260</t>
+        </is>
+      </c>
       <c r="D3" s="4" t="inlineStr"/>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Floor Mat - Pink - Sq Design - 20x32</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr"/>
+          <t>Alco Stay Peg Cabin Hook</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="6" t="n">
-        <v>75</v>
-      </c>
+      <c r="I3" s="6" t="inlineStr"/>
       <c r="J3" s="7" t="n">
         <v>15</v>
       </c>
@@ -686,15 +690,13 @@
         <f>IF(I3="","",I3*(1+J3/100))</f>
         <v/>
       </c>
-      <c r="L3" s="9" t="inlineStr"/>
-      <c r="M3" s="10">
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="9">
         <f>IF(OR(L3="",K3="",L3=0),"",
   (L3-K3)/L3*100)</f>
         <v/>
       </c>
-      <c r="N3" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N3" s="10" t="inlineStr"/>
       <c r="O3" s="4" t="inlineStr"/>
       <c r="P3" s="4" t="inlineStr"/>
       <c r="Q3" s="4" t="inlineStr"/>
@@ -705,30 +707,40 @@
       </c>
       <c r="S3" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
-      <c r="B4" s="12" t="inlineStr"/>
-      <c r="C4" s="12" t="inlineStr"/>
-      <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Floor Mat - Pink - Line Design - 20x32</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr"/>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="inlineStr"/>
-      <c r="I4" s="13" t="n">
-        <v>75</v>
-      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>G239413293</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>13293</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr"/>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Peg Bag</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
       <c r="J4" s="7" t="n">
         <v>15</v>
       </c>
@@ -736,47 +748,57 @@
         <f>IF(I4="","",I4*(1+J4/100))</f>
         <v/>
       </c>
-      <c r="L4" s="9" t="inlineStr"/>
-      <c r="M4" s="10">
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="9">
         <f>IF(OR(L4="",K4="",L4=0),"",
   (L4-K4)/L4*100)</f>
         <v/>
       </c>
-      <c r="N4" s="14" t="inlineStr"/>
-      <c r="O4" s="12" t="inlineStr"/>
-      <c r="P4" s="12" t="inlineStr"/>
-      <c r="Q4" s="12" t="inlineStr"/>
-      <c r="R4" s="12" t="inlineStr">
+      <c r="N4" s="10" t="inlineStr"/>
+      <c r="O4" s="11" t="inlineStr"/>
+      <c r="P4" s="11" t="inlineStr"/>
+      <c r="Q4" s="11" t="inlineStr"/>
+      <c r="R4" s="11" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="S4" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+      <c r="S4" s="11" t="inlineStr">
+        <is>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="4" t="inlineStr"/>
-      <c r="C5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>12RH714003</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>14003</t>
+        </is>
+      </c>
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>FloorMat Striped - l/blue / Beige 21x34</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr"/>
+          <t>Ironing Board Cover</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="6" t="n">
-        <v>100</v>
-      </c>
+      <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="7" t="n">
         <v>15</v>
       </c>
@@ -784,15 +806,13 @@
         <f>IF(I5="","",I5*(1+J5/100))</f>
         <v/>
       </c>
-      <c r="L5" s="9" t="inlineStr"/>
-      <c r="M5" s="10">
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="9">
         <f>IF(OR(L5="",K5="",L5=0),"",
   (L5-K5)/L5*100)</f>
         <v/>
       </c>
-      <c r="N5" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N5" s="10" t="inlineStr"/>
       <c r="O5" s="4" t="inlineStr"/>
       <c r="P5" s="4" t="inlineStr"/>
       <c r="Q5" s="4" t="inlineStr"/>
@@ -803,30 +823,40 @@
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="12" t="inlineStr"/>
-      <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Floor Mat - Striped - Pink Sq Design - 36x60</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr"/>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="inlineStr"/>
-      <c r="I6" s="13" t="n">
-        <v>100</v>
-      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>G239413293-01</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>18234</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Peg Bag - Black/White</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="7" t="n">
         <v>15</v>
       </c>
@@ -834,49 +864,59 @@
         <f>IF(I6="","",I6*(1+J6/100))</f>
         <v/>
       </c>
-      <c r="L6" s="9" t="inlineStr"/>
-      <c r="M6" s="10">
+      <c r="L6" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="M6" s="9">
         <f>IF(OR(L6="",K6="",L6=0),"",
   (L6-K6)/L6*100)</f>
         <v/>
       </c>
-      <c r="N6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="12" t="inlineStr"/>
-      <c r="P6" s="12" t="inlineStr"/>
-      <c r="Q6" s="12" t="inlineStr"/>
-      <c r="R6" s="12" t="inlineStr">
+      <c r="N6" s="10" t="inlineStr"/>
+      <c r="O6" s="11" t="inlineStr"/>
+      <c r="P6" s="11" t="inlineStr"/>
+      <c r="Q6" s="11" t="inlineStr"/>
+      <c r="R6" s="11" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="S6" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+      <c r="S6" s="11" t="inlineStr">
+        <is>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>G239413293-02</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>18235</t>
+        </is>
+      </c>
       <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Floor Mat - Striped - Beige/ Green / Blue - 21 x 34</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr"/>
+          <t>Peg Bag - Navy/White</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="6" t="n">
-        <v>100</v>
-      </c>
+      <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="7" t="n">
         <v>15</v>
       </c>
@@ -884,15 +924,15 @@
         <f>IF(I7="","",I7*(1+J7/100))</f>
         <v/>
       </c>
-      <c r="L7" s="9" t="inlineStr"/>
-      <c r="M7" s="10">
+      <c r="L7" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="M7" s="9">
         <f>IF(OR(L7="",K7="",L7=0),"",
   (L7-K7)/L7*100)</f>
         <v/>
       </c>
-      <c r="N7" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N7" s="10" t="inlineStr"/>
       <c r="O7" s="4" t="inlineStr"/>
       <c r="P7" s="4" t="inlineStr"/>
       <c r="Q7" s="4" t="inlineStr"/>
@@ -903,30 +943,40 @@
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr"/>
-      <c r="B8" s="12" t="inlineStr"/>
-      <c r="C8" s="12" t="inlineStr"/>
-      <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Floor Mat - Striped - Blue/Beige - 21x34</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr"/>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="inlineStr"/>
-      <c r="I8" s="13" t="n">
-        <v>100</v>
-      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>G239413293-03</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>18236</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Peg Bag - Beige/Grey</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="7" t="n">
         <v>15</v>
       </c>
@@ -934,49 +984,59 @@
         <f>IF(I8="","",I8*(1+J8/100))</f>
         <v/>
       </c>
-      <c r="L8" s="9" t="inlineStr"/>
-      <c r="M8" s="10">
+      <c r="L8" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="M8" s="9">
         <f>IF(OR(L8="",K8="",L8=0),"",
   (L8-K8)/L8*100)</f>
         <v/>
       </c>
-      <c r="N8" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="12" t="inlineStr"/>
-      <c r="P8" s="12" t="inlineStr"/>
-      <c r="Q8" s="12" t="inlineStr"/>
-      <c r="R8" s="12" t="inlineStr">
+      <c r="N8" s="10" t="inlineStr"/>
+      <c r="O8" s="11" t="inlineStr"/>
+      <c r="P8" s="11" t="inlineStr"/>
+      <c r="Q8" s="11" t="inlineStr"/>
+      <c r="R8" s="11" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="S8" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+      <c r="S8" s="11" t="inlineStr">
+        <is>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>G239413293-04</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>18237</t>
+        </is>
+      </c>
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Floor Mat - Striped - Pink/Purple - 21x34</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr"/>
+          <t>Peg Bag - Pink/Purple</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="6" t="n">
-        <v>100</v>
-      </c>
+      <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="7" t="n">
         <v>15</v>
       </c>
@@ -984,15 +1044,15 @@
         <f>IF(I9="","",I9*(1+J9/100))</f>
         <v/>
       </c>
-      <c r="L9" s="9" t="inlineStr"/>
-      <c r="M9" s="10">
+      <c r="L9" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="M9" s="9">
         <f>IF(OR(L9="",K9="",L9=0),"",
   (L9-K9)/L9*100)</f>
         <v/>
       </c>
-      <c r="N9" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N9" s="10" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr"/>
       <c r="P9" s="4" t="inlineStr"/>
       <c r="Q9" s="4" t="inlineStr"/>
@@ -1003,30 +1063,40 @@
       </c>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="12" t="inlineStr"/>
-      <c r="C10" s="12" t="inlineStr"/>
-      <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>Floor Mat - Striped - Bright Pink - 17x24 -44/65</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr"/>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="inlineStr"/>
-      <c r="I10" s="13" t="n">
-        <v>60</v>
-      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>G239413293-05</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>18238</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr"/>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Peg Bag - Red/Gold</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="7" t="n">
         <v>15</v>
       </c>
@@ -1034,49 +1104,59 @@
         <f>IF(I10="","",I10*(1+J10/100))</f>
         <v/>
       </c>
-      <c r="L10" s="9" t="inlineStr"/>
-      <c r="M10" s="10">
+      <c r="L10" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="M10" s="9">
         <f>IF(OR(L10="",K10="",L10=0),"",
   (L10-K10)/L10*100)</f>
         <v/>
       </c>
-      <c r="N10" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="12" t="inlineStr"/>
-      <c r="P10" s="12" t="inlineStr"/>
-      <c r="Q10" s="12" t="inlineStr"/>
-      <c r="R10" s="12" t="inlineStr">
+      <c r="N10" s="10" t="inlineStr"/>
+      <c r="O10" s="11" t="inlineStr"/>
+      <c r="P10" s="11" t="inlineStr"/>
+      <c r="Q10" s="11" t="inlineStr"/>
+      <c r="R10" s="11" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="S10" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>12RH714003-01</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>18257</t>
+        </is>
+      </c>
       <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Floor Mat - Striped - Light Pink - 47x75</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr"/>
+          <t>Ironing Board Cover - Pink/White</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="6" t="n">
-        <v>80</v>
-      </c>
+      <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="7" t="n">
         <v>15</v>
       </c>
@@ -1084,15 +1164,15 @@
         <f>IF(I11="","",I11*(1+J11/100))</f>
         <v/>
       </c>
-      <c r="L11" s="9" t="inlineStr"/>
-      <c r="M11" s="10">
+      <c r="L11" s="13" t="n">
+        <v>110</v>
+      </c>
+      <c r="M11" s="9">
         <f>IF(OR(L11="",K11="",L11=0),"",
   (L11-K11)/L11*100)</f>
         <v/>
       </c>
-      <c r="N11" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N11" s="10" t="inlineStr"/>
       <c r="O11" s="4" t="inlineStr"/>
       <c r="P11" s="4" t="inlineStr"/>
       <c r="Q11" s="4" t="inlineStr"/>
@@ -1103,30 +1183,40 @@
       </c>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr"/>
-      <c r="B12" s="12" t="inlineStr"/>
-      <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>Floor Mat - Pattern Rug - red/yellow/blue - 27x45</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr"/>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr"/>
-      <c r="I12" s="13" t="n">
-        <v>180</v>
-      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>12RH714003-02</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>18258</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Ironing Board Cover - Navy/Peach</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="7" t="n">
         <v>15</v>
       </c>
@@ -1134,47 +1224,59 @@
         <f>IF(I12="","",I12*(1+J12/100))</f>
         <v/>
       </c>
-      <c r="L12" s="9" t="inlineStr"/>
-      <c r="M12" s="10">
+      <c r="L12" s="12" t="n">
+        <v>110</v>
+      </c>
+      <c r="M12" s="9">
         <f>IF(OR(L12="",K12="",L12=0),"",
   (L12-K12)/L12*100)</f>
         <v/>
       </c>
-      <c r="N12" s="14" t="inlineStr"/>
-      <c r="O12" s="12" t="inlineStr"/>
-      <c r="P12" s="12" t="inlineStr"/>
-      <c r="Q12" s="12" t="inlineStr"/>
-      <c r="R12" s="12" t="inlineStr">
+      <c r="N12" s="10" t="inlineStr"/>
+      <c r="O12" s="11" t="inlineStr"/>
+      <c r="P12" s="11" t="inlineStr"/>
+      <c r="Q12" s="11" t="inlineStr"/>
+      <c r="R12" s="11" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="S12" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>12RH714003-03</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>18259</t>
+        </is>
+      </c>
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Floor Mat - Red Checked - 21x32</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr"/>
+          <t>Ironing Board Cover - Black/Tri</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="6" t="n">
-        <v>80</v>
-      </c>
+      <c r="I13" s="6" t="inlineStr"/>
       <c r="J13" s="7" t="n">
         <v>15</v>
       </c>
@@ -1182,15 +1284,15 @@
         <f>IF(I13="","",I13*(1+J13/100))</f>
         <v/>
       </c>
-      <c r="L13" s="9" t="inlineStr"/>
-      <c r="M13" s="10">
+      <c r="L13" s="13" t="n">
+        <v>110</v>
+      </c>
+      <c r="M13" s="9">
         <f>IF(OR(L13="",K13="",L13=0),"",
   (L13-K13)/L13*100)</f>
         <v/>
       </c>
-      <c r="N13" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N13" s="10" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
       <c r="P13" s="4" t="inlineStr"/>
       <c r="Q13" s="4" t="inlineStr"/>
@@ -1201,30 +1303,40 @@
       </c>
       <c r="S13" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr"/>
-      <c r="B14" s="12" t="inlineStr"/>
-      <c r="C14" s="12" t="inlineStr"/>
-      <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>Floor Mat - Set 2 - Light Blue - 40x50 + 50x80</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="inlineStr"/>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H14" s="12" t="inlineStr"/>
-      <c r="I14" s="13" t="n">
-        <v>150</v>
-      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>9902056295991-01</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>18802</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr"/>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Alco Stay Peg Cabin Hook - 150mm</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
       <c r="J14" s="7" t="n">
         <v>15</v>
       </c>
@@ -1232,47 +1344,59 @@
         <f>IF(I14="","",I14*(1+J14/100))</f>
         <v/>
       </c>
-      <c r="L14" s="9" t="inlineStr"/>
-      <c r="M14" s="10">
+      <c r="L14" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="M14" s="9">
         <f>IF(OR(L14="",K14="",L14=0),"",
   (L14-K14)/L14*100)</f>
         <v/>
       </c>
-      <c r="N14" s="14" t="inlineStr"/>
-      <c r="O14" s="12" t="inlineStr"/>
-      <c r="P14" s="12" t="inlineStr"/>
-      <c r="Q14" s="12" t="inlineStr"/>
-      <c r="R14" s="12" t="inlineStr">
+      <c r="N14" s="10" t="inlineStr"/>
+      <c r="O14" s="11" t="inlineStr"/>
+      <c r="P14" s="11" t="inlineStr"/>
+      <c r="Q14" s="11" t="inlineStr"/>
+      <c r="R14" s="11" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="S14" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="4" t="inlineStr"/>
-      <c r="C15" s="4" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>9902056295991-02</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>18803</t>
+        </is>
+      </c>
       <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Toilet Mat Set - Pebble Grey Thick - 80x49</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr"/>
+          <t>Alco Stay Peg Cabin Hook - 200mm</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" s="6" t="n">
-        <v>195</v>
-      </c>
+      <c r="I15" s="6" t="inlineStr"/>
       <c r="J15" s="7" t="n">
         <v>15</v>
       </c>
@@ -1280,13 +1404,15 @@
         <f>IF(I15="","",I15*(1+J15/100))</f>
         <v/>
       </c>
-      <c r="L15" s="9" t="inlineStr"/>
-      <c r="M15" s="10">
+      <c r="L15" s="13" t="n">
+        <v>135</v>
+      </c>
+      <c r="M15" s="9">
         <f>IF(OR(L15="",K15="",L15=0),"",
   (L15-K15)/L15*100)</f>
         <v/>
       </c>
-      <c r="N15" s="14" t="inlineStr"/>
+      <c r="N15" s="10" t="inlineStr"/>
       <c r="O15" s="4" t="inlineStr"/>
       <c r="P15" s="4" t="inlineStr"/>
       <c r="Q15" s="4" t="inlineStr"/>
@@ -1297,30 +1423,40 @@
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="12" t="inlineStr"/>
-      <c r="C16" s="12" t="inlineStr"/>
-      <c r="D16" s="12" t="inlineStr"/>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - Floral Blue / Yellow/ Orange Thick - 80x49</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="inlineStr"/>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="inlineStr"/>
-      <c r="I16" s="13" t="n">
-        <v>195</v>
-      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>9902056295991-03</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>18804</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr"/>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Alco Stay Peg Cabin Hook - 250mm</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
       <c r="J16" s="7" t="n">
         <v>15</v>
       </c>
@@ -1328,47 +1464,59 @@
         <f>IF(I16="","",I16*(1+J16/100))</f>
         <v/>
       </c>
-      <c r="L16" s="9" t="inlineStr"/>
-      <c r="M16" s="10">
+      <c r="L16" s="12" t="n">
+        <v>140</v>
+      </c>
+      <c r="M16" s="9">
         <f>IF(OR(L16="",K16="",L16=0),"",
   (L16-K16)/L16*100)</f>
         <v/>
       </c>
-      <c r="N16" s="14" t="inlineStr"/>
-      <c r="O16" s="12" t="inlineStr"/>
-      <c r="P16" s="12" t="inlineStr"/>
-      <c r="Q16" s="12" t="inlineStr"/>
-      <c r="R16" s="12" t="inlineStr">
+      <c r="N16" s="10" t="inlineStr"/>
+      <c r="O16" s="11" t="inlineStr"/>
+      <c r="P16" s="11" t="inlineStr"/>
+      <c r="Q16" s="11" t="inlineStr"/>
+      <c r="R16" s="11" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="S16" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+      <c r="S16" s="11" t="inlineStr">
+        <is>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>9902056295991-04</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>18805</t>
+        </is>
+      </c>
       <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Toilet Mat Set - Beach Vibes - 80x49 - Thick</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr"/>
+          <t>Alco Stay Peg Cabin Hook - 300mm</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Mama Busi</t>
+        </is>
+      </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
+          <t>Homeware</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
-      <c r="I17" s="6" t="n">
-        <v>195</v>
-      </c>
+      <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="7" t="n">
         <v>15</v>
       </c>
@@ -1376,15 +1524,15 @@
         <f>IF(I17="","",I17*(1+J17/100))</f>
         <v/>
       </c>
-      <c r="L17" s="9" t="inlineStr"/>
-      <c r="M17" s="10">
+      <c r="L17" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="M17" s="9">
         <f>IF(OR(L17="",K17="",L17=0),"",
   (L17-K17)/L17*100)</f>
         <v/>
       </c>
-      <c r="N17" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N17" s="10" t="inlineStr"/>
       <c r="O17" s="4" t="inlineStr"/>
       <c r="P17" s="4" t="inlineStr"/>
       <c r="Q17" s="4" t="inlineStr"/>
@@ -1395,30 +1543,20 @@
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
+          <t>Fill in cost price</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="12" t="inlineStr"/>
-      <c r="C18" s="12" t="inlineStr"/>
-      <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - Sleeptime Moon - 80x 49 Thick</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="inlineStr"/>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H18" s="12" t="inlineStr"/>
-      <c r="I18" s="13" t="n">
-        <v>195</v>
-      </c>
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="3" t="n"/>
       <c r="J18" s="7" t="n">
         <v>15</v>
       </c>
@@ -1426,49 +1564,29 @@
         <f>IF(I18="","",I18*(1+J18/100))</f>
         <v/>
       </c>
-      <c r="L18" s="9" t="inlineStr"/>
-      <c r="M18" s="10">
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="9">
         <f>IF(OR(L18="",K18="",L18=0),"",
   (L18-K18)/L18*100)</f>
         <v/>
       </c>
-      <c r="N18" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" s="12" t="inlineStr"/>
-      <c r="P18" s="12" t="inlineStr"/>
-      <c r="Q18" s="12" t="inlineStr"/>
-      <c r="R18" s="12" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="S18" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
-        </is>
-      </c>
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="4" t="n"/>
+      <c r="P18" s="4" t="n"/>
+      <c r="Q18" s="4" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - Light Blue - sea shell star - Thin - 70x45</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="6" t="n">
-        <v>125</v>
-      </c>
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="11" t="n"/>
+      <c r="I19" s="3" t="n"/>
       <c r="J19" s="7" t="n">
         <v>15</v>
       </c>
@@ -1476,49 +1594,29 @@
         <f>IF(I19="","",I19*(1+J19/100))</f>
         <v/>
       </c>
-      <c r="L19" s="9" t="inlineStr"/>
-      <c r="M19" s="10">
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="9">
         <f>IF(OR(L19="",K19="",L19=0),"",
   (L19-K19)/L19*100)</f>
         <v/>
       </c>
-      <c r="N19" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
-      <c r="Q19" s="4" t="inlineStr"/>
-      <c r="R19" s="4" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="S19" s="4" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
-        </is>
-      </c>
+      <c r="N19" s="3" t="n"/>
+      <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="n"/>
+      <c r="Q19" s="11" t="n"/>
+      <c r="R19" s="11" t="n"/>
+      <c r="S19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr"/>
-      <c r="B20" s="12" t="inlineStr"/>
-      <c r="C20" s="12" t="inlineStr"/>
-      <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - Red - Striped - Thin - 70x45</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr"/>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H20" s="12" t="inlineStr"/>
-      <c r="I20" s="13" t="n">
-        <v>125</v>
-      </c>
+      <c r="A20" s="3" t="n"/>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="3" t="n"/>
       <c r="J20" s="7" t="n">
         <v>15</v>
       </c>
@@ -1526,49 +1624,29 @@
         <f>IF(I20="","",I20*(1+J20/100))</f>
         <v/>
       </c>
-      <c r="L20" s="9" t="inlineStr"/>
-      <c r="M20" s="10">
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="9">
         <f>IF(OR(L20="",K20="",L20=0),"",
   (L20-K20)/L20*100)</f>
         <v/>
       </c>
-      <c r="N20" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="12" t="inlineStr"/>
-      <c r="P20" s="12" t="inlineStr"/>
-      <c r="Q20" s="12" t="inlineStr"/>
-      <c r="R20" s="12" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="S20" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
-        </is>
-      </c>
+      <c r="N20" s="3" t="n"/>
+      <c r="O20" s="4" t="n"/>
+      <c r="P20" s="4" t="n"/>
+      <c r="Q20" s="4" t="n"/>
+      <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - Grey Star - Thin - 70x45</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="6" t="n">
-        <v>125</v>
-      </c>
+      <c r="A21" s="3" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="11" t="n"/>
+      <c r="I21" s="3" t="n"/>
       <c r="J21" s="7" t="n">
         <v>15</v>
       </c>
@@ -1576,49 +1654,29 @@
         <f>IF(I21="","",I21*(1+J21/100))</f>
         <v/>
       </c>
-      <c r="L21" s="9" t="inlineStr"/>
-      <c r="M21" s="10">
+      <c r="L21" s="3" t="n"/>
+      <c r="M21" s="9">
         <f>IF(OR(L21="",K21="",L21=0),"",
   (L21-K21)/L21*100)</f>
         <v/>
       </c>
-      <c r="N21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O21" s="4" t="inlineStr"/>
-      <c r="P21" s="4" t="inlineStr"/>
-      <c r="Q21" s="4" t="inlineStr"/>
-      <c r="R21" s="4" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="S21" s="4" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
-        </is>
-      </c>
+      <c r="N21" s="3" t="n"/>
+      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="n"/>
+      <c r="Q21" s="11" t="n"/>
+      <c r="R21" s="11" t="n"/>
+      <c r="S21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="12" t="inlineStr"/>
-      <c r="C22" s="12" t="inlineStr"/>
-      <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - Pebble - Thin - 70x45</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr"/>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H22" s="12" t="inlineStr"/>
-      <c r="I22" s="13" t="n">
-        <v>125</v>
-      </c>
+      <c r="A22" s="3" t="n"/>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="3" t="n"/>
       <c r="J22" s="7" t="n">
         <v>15</v>
       </c>
@@ -1626,49 +1684,29 @@
         <f>IF(I22="","",I22*(1+J22/100))</f>
         <v/>
       </c>
-      <c r="L22" s="9" t="inlineStr"/>
-      <c r="M22" s="10">
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="9">
         <f>IF(OR(L22="",K22="",L22=0),"",
   (L22-K22)/L22*100)</f>
         <v/>
       </c>
-      <c r="N22" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O22" s="12" t="inlineStr"/>
-      <c r="P22" s="12" t="inlineStr"/>
-      <c r="Q22" s="12" t="inlineStr"/>
-      <c r="R22" s="12" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="S22" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
-        </is>
-      </c>
+      <c r="N22" s="3" t="n"/>
+      <c r="O22" s="4" t="n"/>
+      <c r="P22" s="4" t="n"/>
+      <c r="Q22" s="4" t="n"/>
+      <c r="R22" s="4" t="n"/>
+      <c r="S22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr"/>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - Blue Design - Thin - 70x45</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="6" t="n">
-        <v>125</v>
-      </c>
+      <c r="A23" s="3" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="11" t="n"/>
+      <c r="H23" s="11" t="n"/>
+      <c r="I23" s="3" t="n"/>
       <c r="J23" s="7" t="n">
         <v>15</v>
       </c>
@@ -1676,47 +1714,29 @@
         <f>IF(I23="","",I23*(1+J23/100))</f>
         <v/>
       </c>
-      <c r="L23" s="9" t="inlineStr"/>
-      <c r="M23" s="10">
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="9">
         <f>IF(OR(L23="",K23="",L23=0),"",
   (L23-K23)/L23*100)</f>
         <v/>
       </c>
-      <c r="N23" s="14" t="inlineStr"/>
-      <c r="O23" s="4" t="inlineStr"/>
-      <c r="P23" s="4" t="inlineStr"/>
-      <c r="Q23" s="4" t="inlineStr"/>
-      <c r="R23" s="4" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="S23" s="4" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
-        </is>
-      </c>
+      <c r="N23" s="3" t="n"/>
+      <c r="O23" s="11" t="n"/>
+      <c r="P23" s="11" t="n"/>
+      <c r="Q23" s="11" t="n"/>
+      <c r="R23" s="11" t="n"/>
+      <c r="S23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr"/>
-      <c r="B24" s="12" t="inlineStr"/>
-      <c r="C24" s="12" t="inlineStr"/>
-      <c r="D24" s="12" t="inlineStr"/>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>Toilet Mat Set - wood - Thin - 70x45</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr"/>
-      <c r="G24" s="12" t="inlineStr">
-        <is>
-          <t>Homeware &gt; Decor &gt; Carpets</t>
-        </is>
-      </c>
-      <c r="H24" s="12" t="inlineStr"/>
-      <c r="I24" s="13" t="n">
-        <v>125</v>
-      </c>
+      <c r="A24" s="3" t="n"/>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="3" t="n"/>
       <c r="J24" s="7" t="n">
         <v>15</v>
       </c>
@@ -1724,36 +1744,28 @@
         <f>IF(I24="","",I24*(1+J24/100))</f>
         <v/>
       </c>
-      <c r="L24" s="9" t="inlineStr"/>
-      <c r="M24" s="10">
+      <c r="L24" s="3" t="n"/>
+      <c r="M24" s="9">
         <f>IF(OR(L24="",K24="",L24=0),"",
   (L24-K24)/L24*100)</f>
         <v/>
       </c>
-      <c r="N24" s="14" t="inlineStr"/>
-      <c r="O24" s="12" t="inlineStr"/>
-      <c r="P24" s="12" t="inlineStr"/>
-      <c r="Q24" s="12" t="inlineStr"/>
-      <c r="R24" s="12" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="S24" s="12" t="inlineStr">
-        <is>
-          <t>Floor/toilet mat — confirm supplier name</t>
-        </is>
-      </c>
+      <c r="N24" s="3" t="n"/>
+      <c r="O24" s="4" t="n"/>
+      <c r="P24" s="4" t="n"/>
+      <c r="Q24" s="4" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
       <c r="E25" s="3" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="n"/>
+      <c r="H25" s="11" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="7" t="n">
         <v>15</v>
@@ -1763,27 +1775,27 @@
         <v/>
       </c>
       <c r="L25" s="3" t="n"/>
-      <c r="M25" s="10">
+      <c r="M25" s="9">
         <f>IF(OR(L25="",K25="",L25=0),"",
   (L25-K25)/L25*100)</f>
         <v/>
       </c>
       <c r="N25" s="3" t="n"/>
-      <c r="O25" s="4" t="n"/>
-      <c r="P25" s="4" t="n"/>
-      <c r="Q25" s="4" t="n"/>
-      <c r="R25" s="4" t="n"/>
-      <c r="S25" s="4" t="n"/>
+      <c r="O25" s="11" t="n"/>
+      <c r="P25" s="11" t="n"/>
+      <c r="Q25" s="11" t="n"/>
+      <c r="R25" s="11" t="n"/>
+      <c r="S25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
       <c r="E26" s="3" t="n"/>
-      <c r="F26" s="12" t="n"/>
-      <c r="G26" s="12" t="n"/>
-      <c r="H26" s="12" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="7" t="n">
         <v>15</v>
@@ -1793,27 +1805,27 @@
         <v/>
       </c>
       <c r="L26" s="3" t="n"/>
-      <c r="M26" s="10">
+      <c r="M26" s="9">
         <f>IF(OR(L26="",K26="",L26=0),"",
   (L26-K26)/L26*100)</f>
         <v/>
       </c>
       <c r="N26" s="3" t="n"/>
-      <c r="O26" s="12" t="n"/>
-      <c r="P26" s="12" t="n"/>
-      <c r="Q26" s="12" t="n"/>
-      <c r="R26" s="12" t="n"/>
-      <c r="S26" s="12" t="n"/>
+      <c r="O26" s="4" t="n"/>
+      <c r="P26" s="4" t="n"/>
+      <c r="Q26" s="4" t="n"/>
+      <c r="R26" s="4" t="n"/>
+      <c r="S26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
       <c r="E27" s="3" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+      <c r="H27" s="11" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="7" t="n">
         <v>15</v>
@@ -1823,27 +1835,27 @@
         <v/>
       </c>
       <c r="L27" s="3" t="n"/>
-      <c r="M27" s="10">
+      <c r="M27" s="9">
         <f>IF(OR(L27="",K27="",L27=0),"",
   (L27-K27)/L27*100)</f>
         <v/>
       </c>
       <c r="N27" s="3" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
-      <c r="Q27" s="4" t="n"/>
-      <c r="R27" s="4" t="n"/>
-      <c r="S27" s="4" t="n"/>
+      <c r="O27" s="11" t="n"/>
+      <c r="P27" s="11" t="n"/>
+      <c r="Q27" s="11" t="n"/>
+      <c r="R27" s="11" t="n"/>
+      <c r="S27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
       <c r="E28" s="3" t="n"/>
-      <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12" t="n"/>
-      <c r="H28" s="12" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="7" t="n">
         <v>15</v>
@@ -1853,27 +1865,27 @@
         <v/>
       </c>
       <c r="L28" s="3" t="n"/>
-      <c r="M28" s="10">
+      <c r="M28" s="9">
         <f>IF(OR(L28="",K28="",L28=0),"",
   (L28-K28)/L28*100)</f>
         <v/>
       </c>
       <c r="N28" s="3" t="n"/>
-      <c r="O28" s="12" t="n"/>
-      <c r="P28" s="12" t="n"/>
-      <c r="Q28" s="12" t="n"/>
-      <c r="R28" s="12" t="n"/>
-      <c r="S28" s="12" t="n"/>
+      <c r="O28" s="4" t="n"/>
+      <c r="P28" s="4" t="n"/>
+      <c r="Q28" s="4" t="n"/>
+      <c r="R28" s="4" t="n"/>
+      <c r="S28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
       <c r="E29" s="3" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="n"/>
+      <c r="H29" s="11" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="7" t="n">
         <v>15</v>
@@ -1883,27 +1895,27 @@
         <v/>
       </c>
       <c r="L29" s="3" t="n"/>
-      <c r="M29" s="10">
+      <c r="M29" s="9">
         <f>IF(OR(L29="",K29="",L29=0),"",
   (L29-K29)/L29*100)</f>
         <v/>
       </c>
       <c r="N29" s="3" t="n"/>
-      <c r="O29" s="4" t="n"/>
-      <c r="P29" s="4" t="n"/>
-      <c r="Q29" s="4" t="n"/>
-      <c r="R29" s="4" t="n"/>
-      <c r="S29" s="4" t="n"/>
+      <c r="O29" s="11" t="n"/>
+      <c r="P29" s="11" t="n"/>
+      <c r="Q29" s="11" t="n"/>
+      <c r="R29" s="11" t="n"/>
+      <c r="S29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
       <c r="E30" s="3" t="n"/>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="12" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="7" t="n">
         <v>15</v>
@@ -1913,27 +1925,27 @@
         <v/>
       </c>
       <c r="L30" s="3" t="n"/>
-      <c r="M30" s="10">
+      <c r="M30" s="9">
         <f>IF(OR(L30="",K30="",L30=0),"",
   (L30-K30)/L30*100)</f>
         <v/>
       </c>
       <c r="N30" s="3" t="n"/>
-      <c r="O30" s="12" t="n"/>
-      <c r="P30" s="12" t="n"/>
-      <c r="Q30" s="12" t="n"/>
-      <c r="R30" s="12" t="n"/>
-      <c r="S30" s="12" t="n"/>
+      <c r="O30" s="4" t="n"/>
+      <c r="P30" s="4" t="n"/>
+      <c r="Q30" s="4" t="n"/>
+      <c r="R30" s="4" t="n"/>
+      <c r="S30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
       <c r="E31" s="3" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="11" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="7" t="n">
         <v>15</v>
@@ -1943,27 +1955,27 @@
         <v/>
       </c>
       <c r="L31" s="3" t="n"/>
-      <c r="M31" s="10">
+      <c r="M31" s="9">
         <f>IF(OR(L31="",K31="",L31=0),"",
   (L31-K31)/L31*100)</f>
         <v/>
       </c>
       <c r="N31" s="3" t="n"/>
-      <c r="O31" s="4" t="n"/>
-      <c r="P31" s="4" t="n"/>
-      <c r="Q31" s="4" t="n"/>
-      <c r="R31" s="4" t="n"/>
-      <c r="S31" s="4" t="n"/>
+      <c r="O31" s="11" t="n"/>
+      <c r="P31" s="11" t="n"/>
+      <c r="Q31" s="11" t="n"/>
+      <c r="R31" s="11" t="n"/>
+      <c r="S31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="12" t="n"/>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
       <c r="E32" s="3" t="n"/>
-      <c r="F32" s="12" t="n"/>
-      <c r="G32" s="12" t="n"/>
-      <c r="H32" s="12" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="7" t="n">
         <v>15</v>
@@ -1973,27 +1985,27 @@
         <v/>
       </c>
       <c r="L32" s="3" t="n"/>
-      <c r="M32" s="10">
+      <c r="M32" s="9">
         <f>IF(OR(L32="",K32="",L32=0),"",
   (L32-K32)/L32*100)</f>
         <v/>
       </c>
       <c r="N32" s="3" t="n"/>
-      <c r="O32" s="12" t="n"/>
-      <c r="P32" s="12" t="n"/>
-      <c r="Q32" s="12" t="n"/>
-      <c r="R32" s="12" t="n"/>
-      <c r="S32" s="12" t="n"/>
+      <c r="O32" s="4" t="n"/>
+      <c r="P32" s="4" t="n"/>
+      <c r="Q32" s="4" t="n"/>
+      <c r="R32" s="4" t="n"/>
+      <c r="S32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
       <c r="E33" s="3" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
+      <c r="H33" s="11" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="7" t="n">
         <v>15</v>
@@ -2003,27 +2015,27 @@
         <v/>
       </c>
       <c r="L33" s="3" t="n"/>
-      <c r="M33" s="10">
+      <c r="M33" s="9">
         <f>IF(OR(L33="",K33="",L33=0),"",
   (L33-K33)/L33*100)</f>
         <v/>
       </c>
       <c r="N33" s="3" t="n"/>
-      <c r="O33" s="4" t="n"/>
-      <c r="P33" s="4" t="n"/>
-      <c r="Q33" s="4" t="n"/>
-      <c r="R33" s="4" t="n"/>
-      <c r="S33" s="4" t="n"/>
+      <c r="O33" s="11" t="n"/>
+      <c r="P33" s="11" t="n"/>
+      <c r="Q33" s="11" t="n"/>
+      <c r="R33" s="11" t="n"/>
+      <c r="S33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="12" t="n"/>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="n"/>
       <c r="E34" s="3" t="n"/>
-      <c r="F34" s="12" t="n"/>
-      <c r="G34" s="12" t="n"/>
-      <c r="H34" s="12" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="7" t="n">
         <v>15</v>
@@ -2033,27 +2045,27 @@
         <v/>
       </c>
       <c r="L34" s="3" t="n"/>
-      <c r="M34" s="10">
+      <c r="M34" s="9">
         <f>IF(OR(L34="",K34="",L34=0),"",
   (L34-K34)/L34*100)</f>
         <v/>
       </c>
       <c r="N34" s="3" t="n"/>
-      <c r="O34" s="12" t="n"/>
-      <c r="P34" s="12" t="n"/>
-      <c r="Q34" s="12" t="n"/>
-      <c r="R34" s="12" t="n"/>
-      <c r="S34" s="12" t="n"/>
+      <c r="O34" s="4" t="n"/>
+      <c r="P34" s="4" t="n"/>
+      <c r="Q34" s="4" t="n"/>
+      <c r="R34" s="4" t="n"/>
+      <c r="S34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="11" t="n"/>
       <c r="E35" s="3" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="11" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="7" t="n">
         <v>15</v>
@@ -2063,27 +2075,27 @@
         <v/>
       </c>
       <c r="L35" s="3" t="n"/>
-      <c r="M35" s="10">
+      <c r="M35" s="9">
         <f>IF(OR(L35="",K35="",L35=0),"",
   (L35-K35)/L35*100)</f>
         <v/>
       </c>
       <c r="N35" s="3" t="n"/>
-      <c r="O35" s="4" t="n"/>
-      <c r="P35" s="4" t="n"/>
-      <c r="Q35" s="4" t="n"/>
-      <c r="R35" s="4" t="n"/>
-      <c r="S35" s="4" t="n"/>
+      <c r="O35" s="11" t="n"/>
+      <c r="P35" s="11" t="n"/>
+      <c r="Q35" s="11" t="n"/>
+      <c r="R35" s="11" t="n"/>
+      <c r="S35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="12" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
       <c r="E36" s="3" t="n"/>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="12" t="n"/>
-      <c r="H36" s="12" t="n"/>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="7" t="n">
         <v>15</v>
@@ -2093,27 +2105,27 @@
         <v/>
       </c>
       <c r="L36" s="3" t="n"/>
-      <c r="M36" s="10">
+      <c r="M36" s="9">
         <f>IF(OR(L36="",K36="",L36=0),"",
   (L36-K36)/L36*100)</f>
         <v/>
       </c>
       <c r="N36" s="3" t="n"/>
-      <c r="O36" s="12" t="n"/>
-      <c r="P36" s="12" t="n"/>
-      <c r="Q36" s="12" t="n"/>
-      <c r="R36" s="12" t="n"/>
-      <c r="S36" s="12" t="n"/>
+      <c r="O36" s="4" t="n"/>
+      <c r="P36" s="4" t="n"/>
+      <c r="Q36" s="4" t="n"/>
+      <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="11" t="n"/>
       <c r="E37" s="3" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+      <c r="H37" s="11" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="7" t="n">
         <v>15</v>
@@ -2123,27 +2135,27 @@
         <v/>
       </c>
       <c r="L37" s="3" t="n"/>
-      <c r="M37" s="10">
+      <c r="M37" s="9">
         <f>IF(OR(L37="",K37="",L37=0),"",
   (L37-K37)/L37*100)</f>
         <v/>
       </c>
       <c r="N37" s="3" t="n"/>
-      <c r="O37" s="4" t="n"/>
-      <c r="P37" s="4" t="n"/>
-      <c r="Q37" s="4" t="n"/>
-      <c r="R37" s="4" t="n"/>
-      <c r="S37" s="4" t="n"/>
+      <c r="O37" s="11" t="n"/>
+      <c r="P37" s="11" t="n"/>
+      <c r="Q37" s="11" t="n"/>
+      <c r="R37" s="11" t="n"/>
+      <c r="S37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="12" t="n"/>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
       <c r="E38" s="3" t="n"/>
-      <c r="F38" s="12" t="n"/>
-      <c r="G38" s="12" t="n"/>
-      <c r="H38" s="12" t="n"/>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="7" t="n">
         <v>15</v>
@@ -2153,27 +2165,27 @@
         <v/>
       </c>
       <c r="L38" s="3" t="n"/>
-      <c r="M38" s="10">
+      <c r="M38" s="9">
         <f>IF(OR(L38="",K38="",L38=0),"",
   (L38-K38)/L38*100)</f>
         <v/>
       </c>
       <c r="N38" s="3" t="n"/>
-      <c r="O38" s="12" t="n"/>
-      <c r="P38" s="12" t="n"/>
-      <c r="Q38" s="12" t="n"/>
-      <c r="R38" s="12" t="n"/>
-      <c r="S38" s="12" t="n"/>
+      <c r="O38" s="4" t="n"/>
+      <c r="P38" s="4" t="n"/>
+      <c r="Q38" s="4" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
       <c r="E39" s="3" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="11" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="7" t="n">
         <v>15</v>
@@ -2183,27 +2195,27 @@
         <v/>
       </c>
       <c r="L39" s="3" t="n"/>
-      <c r="M39" s="10">
+      <c r="M39" s="9">
         <f>IF(OR(L39="",K39="",L39=0),"",
   (L39-K39)/L39*100)</f>
         <v/>
       </c>
       <c r="N39" s="3" t="n"/>
-      <c r="O39" s="4" t="n"/>
-      <c r="P39" s="4" t="n"/>
-      <c r="Q39" s="4" t="n"/>
-      <c r="R39" s="4" t="n"/>
-      <c r="S39" s="4" t="n"/>
+      <c r="O39" s="11" t="n"/>
+      <c r="P39" s="11" t="n"/>
+      <c r="Q39" s="11" t="n"/>
+      <c r="R39" s="11" t="n"/>
+      <c r="S39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="12" t="n"/>
-      <c r="D40" s="12" t="n"/>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
       <c r="E40" s="3" t="n"/>
-      <c r="F40" s="12" t="n"/>
-      <c r="G40" s="12" t="n"/>
-      <c r="H40" s="12" t="n"/>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="7" t="n">
         <v>15</v>
@@ -2213,27 +2225,27 @@
         <v/>
       </c>
       <c r="L40" s="3" t="n"/>
-      <c r="M40" s="10">
+      <c r="M40" s="9">
         <f>IF(OR(L40="",K40="",L40=0),"",
   (L40-K40)/L40*100)</f>
         <v/>
       </c>
       <c r="N40" s="3" t="n"/>
-      <c r="O40" s="12" t="n"/>
-      <c r="P40" s="12" t="n"/>
-      <c r="Q40" s="12" t="n"/>
-      <c r="R40" s="12" t="n"/>
-      <c r="S40" s="12" t="n"/>
+      <c r="O40" s="4" t="n"/>
+      <c r="P40" s="4" t="n"/>
+      <c r="Q40" s="4" t="n"/>
+      <c r="R40" s="4" t="n"/>
+      <c r="S40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
       <c r="E41" s="3" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="7" t="n">
         <v>15</v>
@@ -2243,27 +2255,27 @@
         <v/>
       </c>
       <c r="L41" s="3" t="n"/>
-      <c r="M41" s="10">
+      <c r="M41" s="9">
         <f>IF(OR(L41="",K41="",L41=0),"",
   (L41-K41)/L41*100)</f>
         <v/>
       </c>
       <c r="N41" s="3" t="n"/>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
-      <c r="Q41" s="4" t="n"/>
-      <c r="R41" s="4" t="n"/>
-      <c r="S41" s="4" t="n"/>
+      <c r="O41" s="11" t="n"/>
+      <c r="P41" s="11" t="n"/>
+      <c r="Q41" s="11" t="n"/>
+      <c r="R41" s="11" t="n"/>
+      <c r="S41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
-      <c r="B42" s="12" t="n"/>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12" t="n"/>
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
       <c r="E42" s="3" t="n"/>
-      <c r="F42" s="12" t="n"/>
-      <c r="G42" s="12" t="n"/>
-      <c r="H42" s="12" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="7" t="n">
         <v>15</v>
@@ -2273,27 +2285,27 @@
         <v/>
       </c>
       <c r="L42" s="3" t="n"/>
-      <c r="M42" s="10">
+      <c r="M42" s="9">
         <f>IF(OR(L42="",K42="",L42=0),"",
   (L42-K42)/L42*100)</f>
         <v/>
       </c>
       <c r="N42" s="3" t="n"/>
-      <c r="O42" s="12" t="n"/>
-      <c r="P42" s="12" t="n"/>
-      <c r="Q42" s="12" t="n"/>
-      <c r="R42" s="12" t="n"/>
-      <c r="S42" s="12" t="n"/>
+      <c r="O42" s="4" t="n"/>
+      <c r="P42" s="4" t="n"/>
+      <c r="Q42" s="4" t="n"/>
+      <c r="R42" s="4" t="n"/>
+      <c r="S42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
+      <c r="B43" s="11" t="n"/>
+      <c r="C43" s="11" t="n"/>
+      <c r="D43" s="11" t="n"/>
       <c r="E43" s="3" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
-      <c r="H43" s="4" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="7" t="n">
         <v>15</v>
@@ -2303,27 +2315,27 @@
         <v/>
       </c>
       <c r="L43" s="3" t="n"/>
-      <c r="M43" s="10">
+      <c r="M43" s="9">
         <f>IF(OR(L43="",K43="",L43=0),"",
   (L43-K43)/L43*100)</f>
         <v/>
       </c>
       <c r="N43" s="3" t="n"/>
-      <c r="O43" s="4" t="n"/>
-      <c r="P43" s="4" t="n"/>
-      <c r="Q43" s="4" t="n"/>
-      <c r="R43" s="4" t="n"/>
-      <c r="S43" s="4" t="n"/>
+      <c r="O43" s="11" t="n"/>
+      <c r="P43" s="11" t="n"/>
+      <c r="Q43" s="11" t="n"/>
+      <c r="R43" s="11" t="n"/>
+      <c r="S43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="n"/>
+      <c r="D44" s="4" t="n"/>
       <c r="E44" s="3" t="n"/>
-      <c r="F44" s="12" t="n"/>
-      <c r="G44" s="12" t="n"/>
-      <c r="H44" s="12" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="7" t="n">
         <v>15</v>
@@ -2333,27 +2345,27 @@
         <v/>
       </c>
       <c r="L44" s="3" t="n"/>
-      <c r="M44" s="10">
+      <c r="M44" s="9">
         <f>IF(OR(L44="",K44="",L44=0),"",
   (L44-K44)/L44*100)</f>
         <v/>
       </c>
       <c r="N44" s="3" t="n"/>
-      <c r="O44" s="12" t="n"/>
-      <c r="P44" s="12" t="n"/>
-      <c r="Q44" s="12" t="n"/>
-      <c r="R44" s="12" t="n"/>
-      <c r="S44" s="12" t="n"/>
+      <c r="O44" s="4" t="n"/>
+      <c r="P44" s="4" t="n"/>
+      <c r="Q44" s="4" t="n"/>
+      <c r="R44" s="4" t="n"/>
+      <c r="S44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
+      <c r="B45" s="11" t="n"/>
+      <c r="C45" s="11" t="n"/>
+      <c r="D45" s="11" t="n"/>
       <c r="E45" s="3" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
-      <c r="H45" s="4" t="n"/>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="11" t="n"/>
+      <c r="H45" s="11" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="7" t="n">
         <v>15</v>
@@ -2363,27 +2375,27 @@
         <v/>
       </c>
       <c r="L45" s="3" t="n"/>
-      <c r="M45" s="10">
+      <c r="M45" s="9">
         <f>IF(OR(L45="",K45="",L45=0),"",
   (L45-K45)/L45*100)</f>
         <v/>
       </c>
       <c r="N45" s="3" t="n"/>
-      <c r="O45" s="4" t="n"/>
-      <c r="P45" s="4" t="n"/>
-      <c r="Q45" s="4" t="n"/>
-      <c r="R45" s="4" t="n"/>
-      <c r="S45" s="4" t="n"/>
+      <c r="O45" s="11" t="n"/>
+      <c r="P45" s="11" t="n"/>
+      <c r="Q45" s="11" t="n"/>
+      <c r="R45" s="11" t="n"/>
+      <c r="S45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="n"/>
+      <c r="D46" s="4" t="n"/>
       <c r="E46" s="3" t="n"/>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-      <c r="H46" s="12" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="7" t="n">
         <v>15</v>
@@ -2393,27 +2405,27 @@
         <v/>
       </c>
       <c r="L46" s="3" t="n"/>
-      <c r="M46" s="10">
+      <c r="M46" s="9">
         <f>IF(OR(L46="",K46="",L46=0),"",
   (L46-K46)/L46*100)</f>
         <v/>
       </c>
       <c r="N46" s="3" t="n"/>
-      <c r="O46" s="12" t="n"/>
-      <c r="P46" s="12" t="n"/>
-      <c r="Q46" s="12" t="n"/>
-      <c r="R46" s="12" t="n"/>
-      <c r="S46" s="12" t="n"/>
+      <c r="O46" s="4" t="n"/>
+      <c r="P46" s="4" t="n"/>
+      <c r="Q46" s="4" t="n"/>
+      <c r="R46" s="4" t="n"/>
+      <c r="S46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
+      <c r="B47" s="11" t="n"/>
+      <c r="C47" s="11" t="n"/>
+      <c r="D47" s="11" t="n"/>
       <c r="E47" s="3" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="4" t="n"/>
-      <c r="H47" s="4" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+      <c r="H47" s="11" t="n"/>
       <c r="I47" s="3" t="n"/>
       <c r="J47" s="7" t="n">
         <v>15</v>
@@ -2423,27 +2435,27 @@
         <v/>
       </c>
       <c r="L47" s="3" t="n"/>
-      <c r="M47" s="10">
+      <c r="M47" s="9">
         <f>IF(OR(L47="",K47="",L47=0),"",
   (L47-K47)/L47*100)</f>
         <v/>
       </c>
       <c r="N47" s="3" t="n"/>
-      <c r="O47" s="4" t="n"/>
-      <c r="P47" s="4" t="n"/>
-      <c r="Q47" s="4" t="n"/>
-      <c r="R47" s="4" t="n"/>
-      <c r="S47" s="4" t="n"/>
+      <c r="O47" s="11" t="n"/>
+      <c r="P47" s="11" t="n"/>
+      <c r="Q47" s="11" t="n"/>
+      <c r="R47" s="11" t="n"/>
+      <c r="S47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
-      <c r="B48" s="12" t="n"/>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="12" t="n"/>
+      <c r="B48" s="4" t="n"/>
+      <c r="C48" s="4" t="n"/>
+      <c r="D48" s="4" t="n"/>
       <c r="E48" s="3" t="n"/>
-      <c r="F48" s="12" t="n"/>
-      <c r="G48" s="12" t="n"/>
-      <c r="H48" s="12" t="n"/>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="7" t="n">
         <v>15</v>
@@ -2453,27 +2465,27 @@
         <v/>
       </c>
       <c r="L48" s="3" t="n"/>
-      <c r="M48" s="10">
+      <c r="M48" s="9">
         <f>IF(OR(L48="",K48="",L48=0),"",
   (L48-K48)/L48*100)</f>
         <v/>
       </c>
       <c r="N48" s="3" t="n"/>
-      <c r="O48" s="12" t="n"/>
-      <c r="P48" s="12" t="n"/>
-      <c r="Q48" s="12" t="n"/>
-      <c r="R48" s="12" t="n"/>
-      <c r="S48" s="12" t="n"/>
+      <c r="O48" s="4" t="n"/>
+      <c r="P48" s="4" t="n"/>
+      <c r="Q48" s="4" t="n"/>
+      <c r="R48" s="4" t="n"/>
+      <c r="S48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
+      <c r="B49" s="11" t="n"/>
+      <c r="C49" s="11" t="n"/>
+      <c r="D49" s="11" t="n"/>
       <c r="E49" s="3" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
-      <c r="H49" s="4" t="n"/>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="11" t="n"/>
+      <c r="H49" s="11" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="7" t="n">
         <v>15</v>
@@ -2483,27 +2495,27 @@
         <v/>
       </c>
       <c r="L49" s="3" t="n"/>
-      <c r="M49" s="10">
+      <c r="M49" s="9">
         <f>IF(OR(L49="",K49="",L49=0),"",
   (L49-K49)/L49*100)</f>
         <v/>
       </c>
       <c r="N49" s="3" t="n"/>
-      <c r="O49" s="4" t="n"/>
-      <c r="P49" s="4" t="n"/>
-      <c r="Q49" s="4" t="n"/>
-      <c r="R49" s="4" t="n"/>
-      <c r="S49" s="4" t="n"/>
+      <c r="O49" s="11" t="n"/>
+      <c r="P49" s="11" t="n"/>
+      <c r="Q49" s="11" t="n"/>
+      <c r="R49" s="11" t="n"/>
+      <c r="S49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
-      <c r="B50" s="12" t="n"/>
-      <c r="C50" s="12" t="n"/>
-      <c r="D50" s="12" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
       <c r="E50" s="3" t="n"/>
-      <c r="F50" s="12" t="n"/>
-      <c r="G50" s="12" t="n"/>
-      <c r="H50" s="12" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="7" t="n">
         <v>15</v>
@@ -2513,27 +2525,27 @@
         <v/>
       </c>
       <c r="L50" s="3" t="n"/>
-      <c r="M50" s="10">
+      <c r="M50" s="9">
         <f>IF(OR(L50="",K50="",L50=0),"",
   (L50-K50)/L50*100)</f>
         <v/>
       </c>
       <c r="N50" s="3" t="n"/>
-      <c r="O50" s="12" t="n"/>
-      <c r="P50" s="12" t="n"/>
-      <c r="Q50" s="12" t="n"/>
-      <c r="R50" s="12" t="n"/>
-      <c r="S50" s="12" t="n"/>
+      <c r="O50" s="4" t="n"/>
+      <c r="P50" s="4" t="n"/>
+      <c r="Q50" s="4" t="n"/>
+      <c r="R50" s="4" t="n"/>
+      <c r="S50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="11" t="n"/>
+      <c r="D51" s="11" t="n"/>
       <c r="E51" s="3" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="11" t="n"/>
+      <c r="H51" s="11" t="n"/>
       <c r="I51" s="3" t="n"/>
       <c r="J51" s="7" t="n">
         <v>15</v>
@@ -2543,27 +2555,27 @@
         <v/>
       </c>
       <c r="L51" s="3" t="n"/>
-      <c r="M51" s="10">
+      <c r="M51" s="9">
         <f>IF(OR(L51="",K51="",L51=0),"",
   (L51-K51)/L51*100)</f>
         <v/>
       </c>
       <c r="N51" s="3" t="n"/>
-      <c r="O51" s="4" t="n"/>
-      <c r="P51" s="4" t="n"/>
-      <c r="Q51" s="4" t="n"/>
-      <c r="R51" s="4" t="n"/>
-      <c r="S51" s="4" t="n"/>
+      <c r="O51" s="11" t="n"/>
+      <c r="P51" s="11" t="n"/>
+      <c r="Q51" s="11" t="n"/>
+      <c r="R51" s="11" t="n"/>
+      <c r="S51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
-      <c r="B52" s="12" t="n"/>
-      <c r="C52" s="12" t="n"/>
-      <c r="D52" s="12" t="n"/>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="4" t="n"/>
+      <c r="D52" s="4" t="n"/>
       <c r="E52" s="3" t="n"/>
-      <c r="F52" s="12" t="n"/>
-      <c r="G52" s="12" t="n"/>
-      <c r="H52" s="12" t="n"/>
+      <c r="F52" s="4" t="n"/>
+      <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="7" t="n">
         <v>15</v>
@@ -2573,27 +2585,27 @@
         <v/>
       </c>
       <c r="L52" s="3" t="n"/>
-      <c r="M52" s="10">
+      <c r="M52" s="9">
         <f>IF(OR(L52="",K52="",L52=0),"",
   (L52-K52)/L52*100)</f>
         <v/>
       </c>
       <c r="N52" s="3" t="n"/>
-      <c r="O52" s="12" t="n"/>
-      <c r="P52" s="12" t="n"/>
-      <c r="Q52" s="12" t="n"/>
-      <c r="R52" s="12" t="n"/>
-      <c r="S52" s="12" t="n"/>
+      <c r="O52" s="4" t="n"/>
+      <c r="P52" s="4" t="n"/>
+      <c r="Q52" s="4" t="n"/>
+      <c r="R52" s="4" t="n"/>
+      <c r="S52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
+      <c r="B53" s="11" t="n"/>
+      <c r="C53" s="11" t="n"/>
+      <c r="D53" s="11" t="n"/>
       <c r="E53" s="3" t="n"/>
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="4" t="n"/>
-      <c r="H53" s="4" t="n"/>
+      <c r="F53" s="11" t="n"/>
+      <c r="G53" s="11" t="n"/>
+      <c r="H53" s="11" t="n"/>
       <c r="I53" s="3" t="n"/>
       <c r="J53" s="7" t="n">
         <v>15</v>
@@ -2603,27 +2615,27 @@
         <v/>
       </c>
       <c r="L53" s="3" t="n"/>
-      <c r="M53" s="10">
+      <c r="M53" s="9">
         <f>IF(OR(L53="",K53="",L53=0),"",
   (L53-K53)/L53*100)</f>
         <v/>
       </c>
       <c r="N53" s="3" t="n"/>
-      <c r="O53" s="4" t="n"/>
-      <c r="P53" s="4" t="n"/>
-      <c r="Q53" s="4" t="n"/>
-      <c r="R53" s="4" t="n"/>
-      <c r="S53" s="4" t="n"/>
+      <c r="O53" s="11" t="n"/>
+      <c r="P53" s="11" t="n"/>
+      <c r="Q53" s="11" t="n"/>
+      <c r="R53" s="11" t="n"/>
+      <c r="S53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
-      <c r="B54" s="12" t="n"/>
-      <c r="C54" s="12" t="n"/>
-      <c r="D54" s="12" t="n"/>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="4" t="n"/>
       <c r="E54" s="3" t="n"/>
-      <c r="F54" s="12" t="n"/>
-      <c r="G54" s="12" t="n"/>
-      <c r="H54" s="12" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="7" t="n">
         <v>15</v>
@@ -2633,27 +2645,27 @@
         <v/>
       </c>
       <c r="L54" s="3" t="n"/>
-      <c r="M54" s="10">
+      <c r="M54" s="9">
         <f>IF(OR(L54="",K54="",L54=0),"",
   (L54-K54)/L54*100)</f>
         <v/>
       </c>
       <c r="N54" s="3" t="n"/>
-      <c r="O54" s="12" t="n"/>
-      <c r="P54" s="12" t="n"/>
-      <c r="Q54" s="12" t="n"/>
-      <c r="R54" s="12" t="n"/>
-      <c r="S54" s="12" t="n"/>
+      <c r="O54" s="4" t="n"/>
+      <c r="P54" s="4" t="n"/>
+      <c r="Q54" s="4" t="n"/>
+      <c r="R54" s="4" t="n"/>
+      <c r="S54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="11" t="n"/>
       <c r="E55" s="3" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="4" t="n"/>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="11" t="n"/>
+      <c r="H55" s="11" t="n"/>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="7" t="n">
         <v>15</v>
@@ -2663,27 +2675,27 @@
         <v/>
       </c>
       <c r="L55" s="3" t="n"/>
-      <c r="M55" s="10">
+      <c r="M55" s="9">
         <f>IF(OR(L55="",K55="",L55=0),"",
   (L55-K55)/L55*100)</f>
         <v/>
       </c>
       <c r="N55" s="3" t="n"/>
-      <c r="O55" s="4" t="n"/>
-      <c r="P55" s="4" t="n"/>
-      <c r="Q55" s="4" t="n"/>
-      <c r="R55" s="4" t="n"/>
-      <c r="S55" s="4" t="n"/>
+      <c r="O55" s="11" t="n"/>
+      <c r="P55" s="11" t="n"/>
+      <c r="Q55" s="11" t="n"/>
+      <c r="R55" s="11" t="n"/>
+      <c r="S55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
-      <c r="B56" s="12" t="n"/>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="12" t="n"/>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
       <c r="E56" s="3" t="n"/>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="12" t="n"/>
-      <c r="H56" s="12" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
       <c r="I56" s="3" t="n"/>
       <c r="J56" s="7" t="n">
         <v>15</v>
@@ -2693,27 +2705,27 @@
         <v/>
       </c>
       <c r="L56" s="3" t="n"/>
-      <c r="M56" s="10">
+      <c r="M56" s="9">
         <f>IF(OR(L56="",K56="",L56=0),"",
   (L56-K56)/L56*100)</f>
         <v/>
       </c>
       <c r="N56" s="3" t="n"/>
-      <c r="O56" s="12" t="n"/>
-      <c r="P56" s="12" t="n"/>
-      <c r="Q56" s="12" t="n"/>
-      <c r="R56" s="12" t="n"/>
-      <c r="S56" s="12" t="n"/>
+      <c r="O56" s="4" t="n"/>
+      <c r="P56" s="4" t="n"/>
+      <c r="Q56" s="4" t="n"/>
+      <c r="R56" s="4" t="n"/>
+      <c r="S56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="4" t="n"/>
+      <c r="B57" s="11" t="n"/>
+      <c r="C57" s="11" t="n"/>
+      <c r="D57" s="11" t="n"/>
       <c r="E57" s="3" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
-      <c r="H57" s="4" t="n"/>
+      <c r="F57" s="11" t="n"/>
+      <c r="G57" s="11" t="n"/>
+      <c r="H57" s="11" t="n"/>
       <c r="I57" s="3" t="n"/>
       <c r="J57" s="7" t="n">
         <v>15</v>
@@ -2723,27 +2735,27 @@
         <v/>
       </c>
       <c r="L57" s="3" t="n"/>
-      <c r="M57" s="10">
+      <c r="M57" s="9">
         <f>IF(OR(L57="",K57="",L57=0),"",
   (L57-K57)/L57*100)</f>
         <v/>
       </c>
       <c r="N57" s="3" t="n"/>
-      <c r="O57" s="4" t="n"/>
-      <c r="P57" s="4" t="n"/>
-      <c r="Q57" s="4" t="n"/>
-      <c r="R57" s="4" t="n"/>
-      <c r="S57" s="4" t="n"/>
+      <c r="O57" s="11" t="n"/>
+      <c r="P57" s="11" t="n"/>
+      <c r="Q57" s="11" t="n"/>
+      <c r="R57" s="11" t="n"/>
+      <c r="S57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="4" t="n"/>
+      <c r="D58" s="4" t="n"/>
       <c r="E58" s="3" t="n"/>
-      <c r="F58" s="12" t="n"/>
-      <c r="G58" s="12" t="n"/>
-      <c r="H58" s="12" t="n"/>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
       <c r="I58" s="3" t="n"/>
       <c r="J58" s="7" t="n">
         <v>15</v>
@@ -2753,27 +2765,27 @@
         <v/>
       </c>
       <c r="L58" s="3" t="n"/>
-      <c r="M58" s="10">
+      <c r="M58" s="9">
         <f>IF(OR(L58="",K58="",L58=0),"",
   (L58-K58)/L58*100)</f>
         <v/>
       </c>
       <c r="N58" s="3" t="n"/>
-      <c r="O58" s="12" t="n"/>
-      <c r="P58" s="12" t="n"/>
-      <c r="Q58" s="12" t="n"/>
-      <c r="R58" s="12" t="n"/>
-      <c r="S58" s="12" t="n"/>
+      <c r="O58" s="4" t="n"/>
+      <c r="P58" s="4" t="n"/>
+      <c r="Q58" s="4" t="n"/>
+      <c r="R58" s="4" t="n"/>
+      <c r="S58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
+      <c r="B59" s="11" t="n"/>
+      <c r="C59" s="11" t="n"/>
+      <c r="D59" s="11" t="n"/>
       <c r="E59" s="3" t="n"/>
-      <c r="F59" s="4" t="n"/>
-      <c r="G59" s="4" t="n"/>
-      <c r="H59" s="4" t="n"/>
+      <c r="F59" s="11" t="n"/>
+      <c r="G59" s="11" t="n"/>
+      <c r="H59" s="11" t="n"/>
       <c r="I59" s="3" t="n"/>
       <c r="J59" s="7" t="n">
         <v>15</v>
@@ -2783,27 +2795,27 @@
         <v/>
       </c>
       <c r="L59" s="3" t="n"/>
-      <c r="M59" s="10">
+      <c r="M59" s="9">
         <f>IF(OR(L59="",K59="",L59=0),"",
   (L59-K59)/L59*100)</f>
         <v/>
       </c>
       <c r="N59" s="3" t="n"/>
-      <c r="O59" s="4" t="n"/>
-      <c r="P59" s="4" t="n"/>
-      <c r="Q59" s="4" t="n"/>
-      <c r="R59" s="4" t="n"/>
-      <c r="S59" s="4" t="n"/>
+      <c r="O59" s="11" t="n"/>
+      <c r="P59" s="11" t="n"/>
+      <c r="Q59" s="11" t="n"/>
+      <c r="R59" s="11" t="n"/>
+      <c r="S59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
-      <c r="B60" s="12" t="n"/>
-      <c r="C60" s="12" t="n"/>
-      <c r="D60" s="12" t="n"/>
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="n"/>
+      <c r="D60" s="4" t="n"/>
       <c r="E60" s="3" t="n"/>
-      <c r="F60" s="12" t="n"/>
-      <c r="G60" s="12" t="n"/>
-      <c r="H60" s="12" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
       <c r="I60" s="3" t="n"/>
       <c r="J60" s="7" t="n">
         <v>15</v>
@@ -2813,27 +2825,27 @@
         <v/>
       </c>
       <c r="L60" s="3" t="n"/>
-      <c r="M60" s="10">
+      <c r="M60" s="9">
         <f>IF(OR(L60="",K60="",L60=0),"",
   (L60-K60)/L60*100)</f>
         <v/>
       </c>
       <c r="N60" s="3" t="n"/>
-      <c r="O60" s="12" t="n"/>
-      <c r="P60" s="12" t="n"/>
-      <c r="Q60" s="12" t="n"/>
-      <c r="R60" s="12" t="n"/>
-      <c r="S60" s="12" t="n"/>
+      <c r="O60" s="4" t="n"/>
+      <c r="P60" s="4" t="n"/>
+      <c r="Q60" s="4" t="n"/>
+      <c r="R60" s="4" t="n"/>
+      <c r="S60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="4" t="n"/>
+      <c r="B61" s="11" t="n"/>
+      <c r="C61" s="11" t="n"/>
+      <c r="D61" s="11" t="n"/>
       <c r="E61" s="3" t="n"/>
-      <c r="F61" s="4" t="n"/>
-      <c r="G61" s="4" t="n"/>
-      <c r="H61" s="4" t="n"/>
+      <c r="F61" s="11" t="n"/>
+      <c r="G61" s="11" t="n"/>
+      <c r="H61" s="11" t="n"/>
       <c r="I61" s="3" t="n"/>
       <c r="J61" s="7" t="n">
         <v>15</v>
@@ -2843,27 +2855,27 @@
         <v/>
       </c>
       <c r="L61" s="3" t="n"/>
-      <c r="M61" s="10">
+      <c r="M61" s="9">
         <f>IF(OR(L61="",K61="",L61=0),"",
   (L61-K61)/L61*100)</f>
         <v/>
       </c>
       <c r="N61" s="3" t="n"/>
-      <c r="O61" s="4" t="n"/>
-      <c r="P61" s="4" t="n"/>
-      <c r="Q61" s="4" t="n"/>
-      <c r="R61" s="4" t="n"/>
-      <c r="S61" s="4" t="n"/>
+      <c r="O61" s="11" t="n"/>
+      <c r="P61" s="11" t="n"/>
+      <c r="Q61" s="11" t="n"/>
+      <c r="R61" s="11" t="n"/>
+      <c r="S61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
-      <c r="B62" s="12" t="n"/>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="12" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="4" t="n"/>
+      <c r="D62" s="4" t="n"/>
       <c r="E62" s="3" t="n"/>
-      <c r="F62" s="12" t="n"/>
-      <c r="G62" s="12" t="n"/>
-      <c r="H62" s="12" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
       <c r="I62" s="3" t="n"/>
       <c r="J62" s="7" t="n">
         <v>15</v>
@@ -2873,27 +2885,27 @@
         <v/>
       </c>
       <c r="L62" s="3" t="n"/>
-      <c r="M62" s="10">
+      <c r="M62" s="9">
         <f>IF(OR(L62="",K62="",L62=0),"",
   (L62-K62)/L62*100)</f>
         <v/>
       </c>
       <c r="N62" s="3" t="n"/>
-      <c r="O62" s="12" t="n"/>
-      <c r="P62" s="12" t="n"/>
-      <c r="Q62" s="12" t="n"/>
-      <c r="R62" s="12" t="n"/>
-      <c r="S62" s="12" t="n"/>
+      <c r="O62" s="4" t="n"/>
+      <c r="P62" s="4" t="n"/>
+      <c r="Q62" s="4" t="n"/>
+      <c r="R62" s="4" t="n"/>
+      <c r="S62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="4" t="n"/>
+      <c r="B63" s="11" t="n"/>
+      <c r="C63" s="11" t="n"/>
+      <c r="D63" s="11" t="n"/>
       <c r="E63" s="3" t="n"/>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
-      <c r="H63" s="4" t="n"/>
+      <c r="F63" s="11" t="n"/>
+      <c r="G63" s="11" t="n"/>
+      <c r="H63" s="11" t="n"/>
       <c r="I63" s="3" t="n"/>
       <c r="J63" s="7" t="n">
         <v>15</v>
@@ -2903,27 +2915,27 @@
         <v/>
       </c>
       <c r="L63" s="3" t="n"/>
-      <c r="M63" s="10">
+      <c r="M63" s="9">
         <f>IF(OR(L63="",K63="",L63=0),"",
   (L63-K63)/L63*100)</f>
         <v/>
       </c>
       <c r="N63" s="3" t="n"/>
-      <c r="O63" s="4" t="n"/>
-      <c r="P63" s="4" t="n"/>
-      <c r="Q63" s="4" t="n"/>
-      <c r="R63" s="4" t="n"/>
-      <c r="S63" s="4" t="n"/>
+      <c r="O63" s="11" t="n"/>
+      <c r="P63" s="11" t="n"/>
+      <c r="Q63" s="11" t="n"/>
+      <c r="R63" s="11" t="n"/>
+      <c r="S63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
-      <c r="B64" s="12" t="n"/>
-      <c r="C64" s="12" t="n"/>
-      <c r="D64" s="12" t="n"/>
+      <c r="B64" s="4" t="n"/>
+      <c r="C64" s="4" t="n"/>
+      <c r="D64" s="4" t="n"/>
       <c r="E64" s="3" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="12" t="n"/>
-      <c r="H64" s="12" t="n"/>
+      <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="n"/>
       <c r="I64" s="3" t="n"/>
       <c r="J64" s="7" t="n">
         <v>15</v>
@@ -2933,27 +2945,27 @@
         <v/>
       </c>
       <c r="L64" s="3" t="n"/>
-      <c r="M64" s="10">
+      <c r="M64" s="9">
         <f>IF(OR(L64="",K64="",L64=0),"",
   (L64-K64)/L64*100)</f>
         <v/>
       </c>
       <c r="N64" s="3" t="n"/>
-      <c r="O64" s="12" t="n"/>
-      <c r="P64" s="12" t="n"/>
-      <c r="Q64" s="12" t="n"/>
-      <c r="R64" s="12" t="n"/>
-      <c r="S64" s="12" t="n"/>
+      <c r="O64" s="4" t="n"/>
+      <c r="P64" s="4" t="n"/>
+      <c r="Q64" s="4" t="n"/>
+      <c r="R64" s="4" t="n"/>
+      <c r="S64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
-      <c r="B65" s="4" t="n"/>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="4" t="n"/>
+      <c r="B65" s="11" t="n"/>
+      <c r="C65" s="11" t="n"/>
+      <c r="D65" s="11" t="n"/>
       <c r="E65" s="3" t="n"/>
-      <c r="F65" s="4" t="n"/>
-      <c r="G65" s="4" t="n"/>
-      <c r="H65" s="4" t="n"/>
+      <c r="F65" s="11" t="n"/>
+      <c r="G65" s="11" t="n"/>
+      <c r="H65" s="11" t="n"/>
       <c r="I65" s="3" t="n"/>
       <c r="J65" s="7" t="n">
         <v>15</v>
@@ -2963,27 +2975,27 @@
         <v/>
       </c>
       <c r="L65" s="3" t="n"/>
-      <c r="M65" s="10">
+      <c r="M65" s="9">
         <f>IF(OR(L65="",K65="",L65=0),"",
   (L65-K65)/L65*100)</f>
         <v/>
       </c>
       <c r="N65" s="3" t="n"/>
-      <c r="O65" s="4" t="n"/>
-      <c r="P65" s="4" t="n"/>
-      <c r="Q65" s="4" t="n"/>
-      <c r="R65" s="4" t="n"/>
-      <c r="S65" s="4" t="n"/>
+      <c r="O65" s="11" t="n"/>
+      <c r="P65" s="11" t="n"/>
+      <c r="Q65" s="11" t="n"/>
+      <c r="R65" s="11" t="n"/>
+      <c r="S65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
-      <c r="B66" s="12" t="n"/>
-      <c r="C66" s="12" t="n"/>
-      <c r="D66" s="12" t="n"/>
+      <c r="B66" s="4" t="n"/>
+      <c r="C66" s="4" t="n"/>
+      <c r="D66" s="4" t="n"/>
       <c r="E66" s="3" t="n"/>
-      <c r="F66" s="12" t="n"/>
-      <c r="G66" s="12" t="n"/>
-      <c r="H66" s="12" t="n"/>
+      <c r="F66" s="4" t="n"/>
+      <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="n"/>
       <c r="I66" s="3" t="n"/>
       <c r="J66" s="7" t="n">
         <v>15</v>
@@ -2993,27 +3005,27 @@
         <v/>
       </c>
       <c r="L66" s="3" t="n"/>
-      <c r="M66" s="10">
+      <c r="M66" s="9">
         <f>IF(OR(L66="",K66="",L66=0),"",
   (L66-K66)/L66*100)</f>
         <v/>
       </c>
       <c r="N66" s="3" t="n"/>
-      <c r="O66" s="12" t="n"/>
-      <c r="P66" s="12" t="n"/>
-      <c r="Q66" s="12" t="n"/>
-      <c r="R66" s="12" t="n"/>
-      <c r="S66" s="12" t="n"/>
+      <c r="O66" s="4" t="n"/>
+      <c r="P66" s="4" t="n"/>
+      <c r="Q66" s="4" t="n"/>
+      <c r="R66" s="4" t="n"/>
+      <c r="S66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
-      <c r="B67" s="4" t="n"/>
-      <c r="C67" s="4" t="n"/>
-      <c r="D67" s="4" t="n"/>
+      <c r="B67" s="11" t="n"/>
+      <c r="C67" s="11" t="n"/>
+      <c r="D67" s="11" t="n"/>
       <c r="E67" s="3" t="n"/>
-      <c r="F67" s="4" t="n"/>
-      <c r="G67" s="4" t="n"/>
-      <c r="H67" s="4" t="n"/>
+      <c r="F67" s="11" t="n"/>
+      <c r="G67" s="11" t="n"/>
+      <c r="H67" s="11" t="n"/>
       <c r="I67" s="3" t="n"/>
       <c r="J67" s="7" t="n">
         <v>15</v>
@@ -3023,227 +3035,17 @@
         <v/>
       </c>
       <c r="L67" s="3" t="n"/>
-      <c r="M67" s="10">
+      <c r="M67" s="9">
         <f>IF(OR(L67="",K67="",L67=0),"",
   (L67-K67)/L67*100)</f>
         <v/>
       </c>
       <c r="N67" s="3" t="n"/>
-      <c r="O67" s="4" t="n"/>
-      <c r="P67" s="4" t="n"/>
-      <c r="Q67" s="4" t="n"/>
-      <c r="R67" s="4" t="n"/>
-      <c r="S67" s="4" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="n"/>
-      <c r="B68" s="12" t="n"/>
-      <c r="C68" s="12" t="n"/>
-      <c r="D68" s="12" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="12" t="n"/>
-      <c r="G68" s="12" t="n"/>
-      <c r="H68" s="12" t="n"/>
-      <c r="I68" s="3" t="n"/>
-      <c r="J68" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="K68" s="8">
-        <f>IF(I68="","",I68*(1+J68/100))</f>
-        <v/>
-      </c>
-      <c r="L68" s="3" t="n"/>
-      <c r="M68" s="10">
-        <f>IF(OR(L68="",K68="",L68=0),"",
-  (L68-K68)/L68*100)</f>
-        <v/>
-      </c>
-      <c r="N68" s="3" t="n"/>
-      <c r="O68" s="12" t="n"/>
-      <c r="P68" s="12" t="n"/>
-      <c r="Q68" s="12" t="n"/>
-      <c r="R68" s="12" t="n"/>
-      <c r="S68" s="12" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="n"/>
-      <c r="B69" s="4" t="n"/>
-      <c r="C69" s="4" t="n"/>
-      <c r="D69" s="4" t="n"/>
-      <c r="E69" s="3" t="n"/>
-      <c r="F69" s="4" t="n"/>
-      <c r="G69" s="4" t="n"/>
-      <c r="H69" s="4" t="n"/>
-      <c r="I69" s="3" t="n"/>
-      <c r="J69" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="K69" s="8">
-        <f>IF(I69="","",I69*(1+J69/100))</f>
-        <v/>
-      </c>
-      <c r="L69" s="3" t="n"/>
-      <c r="M69" s="10">
-        <f>IF(OR(L69="",K69="",L69=0),"",
-  (L69-K69)/L69*100)</f>
-        <v/>
-      </c>
-      <c r="N69" s="3" t="n"/>
-      <c r="O69" s="4" t="n"/>
-      <c r="P69" s="4" t="n"/>
-      <c r="Q69" s="4" t="n"/>
-      <c r="R69" s="4" t="n"/>
-      <c r="S69" s="4" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="n"/>
-      <c r="B70" s="12" t="n"/>
-      <c r="C70" s="12" t="n"/>
-      <c r="D70" s="12" t="n"/>
-      <c r="E70" s="3" t="n"/>
-      <c r="F70" s="12" t="n"/>
-      <c r="G70" s="12" t="n"/>
-      <c r="H70" s="12" t="n"/>
-      <c r="I70" s="3" t="n"/>
-      <c r="J70" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="K70" s="8">
-        <f>IF(I70="","",I70*(1+J70/100))</f>
-        <v/>
-      </c>
-      <c r="L70" s="3" t="n"/>
-      <c r="M70" s="10">
-        <f>IF(OR(L70="",K70="",L70=0),"",
-  (L70-K70)/L70*100)</f>
-        <v/>
-      </c>
-      <c r="N70" s="3" t="n"/>
-      <c r="O70" s="12" t="n"/>
-      <c r="P70" s="12" t="n"/>
-      <c r="Q70" s="12" t="n"/>
-      <c r="R70" s="12" t="n"/>
-      <c r="S70" s="12" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="n"/>
-      <c r="B71" s="4" t="n"/>
-      <c r="C71" s="4" t="n"/>
-      <c r="D71" s="4" t="n"/>
-      <c r="E71" s="3" t="n"/>
-      <c r="F71" s="4" t="n"/>
-      <c r="G71" s="4" t="n"/>
-      <c r="H71" s="4" t="n"/>
-      <c r="I71" s="3" t="n"/>
-      <c r="J71" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="K71" s="8">
-        <f>IF(I71="","",I71*(1+J71/100))</f>
-        <v/>
-      </c>
-      <c r="L71" s="3" t="n"/>
-      <c r="M71" s="10">
-        <f>IF(OR(L71="",K71="",L71=0),"",
-  (L71-K71)/L71*100)</f>
-        <v/>
-      </c>
-      <c r="N71" s="3" t="n"/>
-      <c r="O71" s="4" t="n"/>
-      <c r="P71" s="4" t="n"/>
-      <c r="Q71" s="4" t="n"/>
-      <c r="R71" s="4" t="n"/>
-      <c r="S71" s="4" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="n"/>
-      <c r="B72" s="12" t="n"/>
-      <c r="C72" s="12" t="n"/>
-      <c r="D72" s="12" t="n"/>
-      <c r="E72" s="3" t="n"/>
-      <c r="F72" s="12" t="n"/>
-      <c r="G72" s="12" t="n"/>
-      <c r="H72" s="12" t="n"/>
-      <c r="I72" s="3" t="n"/>
-      <c r="J72" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="K72" s="8">
-        <f>IF(I72="","",I72*(1+J72/100))</f>
-        <v/>
-      </c>
-      <c r="L72" s="3" t="n"/>
-      <c r="M72" s="10">
-        <f>IF(OR(L72="",K72="",L72=0),"",
-  (L72-K72)/L72*100)</f>
-        <v/>
-      </c>
-      <c r="N72" s="3" t="n"/>
-      <c r="O72" s="12" t="n"/>
-      <c r="P72" s="12" t="n"/>
-      <c r="Q72" s="12" t="n"/>
-      <c r="R72" s="12" t="n"/>
-      <c r="S72" s="12" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="n"/>
-      <c r="B73" s="4" t="n"/>
-      <c r="C73" s="4" t="n"/>
-      <c r="D73" s="4" t="n"/>
-      <c r="E73" s="3" t="n"/>
-      <c r="F73" s="4" t="n"/>
-      <c r="G73" s="4" t="n"/>
-      <c r="H73" s="4" t="n"/>
-      <c r="I73" s="3" t="n"/>
-      <c r="J73" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="K73" s="8">
-        <f>IF(I73="","",I73*(1+J73/100))</f>
-        <v/>
-      </c>
-      <c r="L73" s="3" t="n"/>
-      <c r="M73" s="10">
-        <f>IF(OR(L73="",K73="",L73=0),"",
-  (L73-K73)/L73*100)</f>
-        <v/>
-      </c>
-      <c r="N73" s="3" t="n"/>
-      <c r="O73" s="4" t="n"/>
-      <c r="P73" s="4" t="n"/>
-      <c r="Q73" s="4" t="n"/>
-      <c r="R73" s="4" t="n"/>
-      <c r="S73" s="4" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="3" t="n"/>
-      <c r="B74" s="12" t="n"/>
-      <c r="C74" s="12" t="n"/>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="3" t="n"/>
-      <c r="F74" s="12" t="n"/>
-      <c r="G74" s="12" t="n"/>
-      <c r="H74" s="12" t="n"/>
-      <c r="I74" s="3" t="n"/>
-      <c r="J74" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="K74" s="8">
-        <f>IF(I74="","",I74*(1+J74/100))</f>
-        <v/>
-      </c>
-      <c r="L74" s="3" t="n"/>
-      <c r="M74" s="10">
-        <f>IF(OR(L74="",K74="",L74=0),"",
-  (L74-K74)/L74*100)</f>
-        <v/>
-      </c>
-      <c r="N74" s="3" t="n"/>
-      <c r="O74" s="12" t="n"/>
-      <c r="P74" s="12" t="n"/>
-      <c r="Q74" s="12" t="n"/>
-      <c r="R74" s="12" t="n"/>
-      <c r="S74" s="12" t="n"/>
+      <c r="O67" s="11" t="n"/>
+      <c r="P67" s="11" t="n"/>
+      <c r="Q67" s="11" t="n"/>
+      <c r="R67" s="11" t="n"/>
+      <c r="S67" s="11" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:S2"/>
@@ -3268,282 +3070,282 @@
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>COLOUR KEY</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr"/>
+      <c r="B1" s="15" t="inlineStr"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Orange background</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Required field — must be filled in</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Yellow background</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Auto-calculated — do not edit manually</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Blue tint rows</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Alternating row shading for readability</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="18" t="inlineStr"/>
-      <c r="B5" s="17" t="inlineStr"/>
+      <c r="A5" s="16" t="inlineStr"/>
+      <c r="B5" s="15" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>COLUMN GUIDE</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr"/>
+      <c r="B6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Supplier SKU</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Supplier's own product code</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>WC SKU</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>WooCommerce SKU (auto-matched)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>WC ID</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>WooCommerce product ID</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Barcode / EAN</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>EAN-13, UPC or internal barcode</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Product Name</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Full product name as it appears on the store</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Brand / manufacturer</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>e.g. Homeware &gt; Kitchenware</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Short product description</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Cost Price (ex VAT)</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>What you pay the supplier, before VAT (R)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>VAT Rate %</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>0 or 15 (auto-applied below)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Cost Price (incl VAT)</t>
         </is>
       </c>
-      <c r="B17" s="17">
+      <c r="B17" s="15">
         <f>Cost*(1+VAT/100) — auto-calculated</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Selling Price (R)</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Your retail price including VAT</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Margin %</t>
         </is>
       </c>
-      <c r="B19" s="17">
+      <c r="B19" s="15">
         <f>(Selling-Cost_incl)/Selling*100 — auto</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Qty On Hand</t>
         </is>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Current physical stock count</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Reorder Level</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Alert when stock falls below this number</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Location / Bay</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Shelf, bay or bin reference in store</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Image URL</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Direct URL or Drive link to product image</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Date this row was last updated</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Any supplier notes, variants, issues</t>
         </is>

</xml_diff>